<commit_message>
73212: remove stale GAP rows (backups were filed); rebuild register
The 73212 evidence manifest carried two stale "unsighted" GAP rows for the
GJ079210 ($66,183.82) and GJ076924 ($1,914) backups alongside the actual SIGHTED
rows for the same items (NA73212_L06/L07 DocLineTables, filed with SHA-256). The
register was correct - both CLOSED 11-Jun, balanced and direction-verified - so
the GAP placeholders were stale leftovers from before the backups were filed.
Removed them. Outstanding Lines Register rebuilt: EVIDENCE 25->23, 73212 now shows
only its two genuine gaps (s4090230 vendor invoices, $20k-floor contracts).
Handover correction note added; manifest regenerated, strict verify PASS.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E2DraJoXMLMxk1NyzJ13Vc
</commit_message>
<xml_diff>
--- a/00_Outstanding_Lines_Register.xlsx
+++ b/00_Outstanding_Lines_Register.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -495,7 +495,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LCC Parks 4090000 - OPEN ACTIONS (rebuilt 18-Jun: live journal + Decisions list + evidence-manifest GAP rows; filed/closed items excluded)</t>
+          <t>LCC Parks 4090000 - OPEN ACTIONS (rebuilt 18-Jun: live journal + Decisions + evidence-manifest GAP rows; filed/closed excluded)</t>
         </is>
       </c>
     </row>
@@ -1520,14 +1520,10 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Sight/obtain: GJ079210 backup (Play Force move)</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>66183.82</t>
-        </is>
-      </c>
+          <t>Sight/obtain: s4090230 standing-order vendor invoices</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr"/>
       <c r="E42" s="4" t="inlineStr">
         <is>
           <t>NA73212_Evidence_Manifest.csv</t>
@@ -1547,7 +1543,7 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Sight/obtain: s4090230 standing-order vendor invoices</t>
+          <t>Sight/obtain: Contracts: LCC-09-2022, Aust Care SO, Play Force</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr"/>
@@ -1565,22 +1561,22 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>73212</t>
+          <t>73511</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Sight/obtain: GJ076924 backup</t>
+          <t>Sight/obtain: INV-9747</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>1914.00</t>
+          <t>2445.45</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>NA73212_Evidence_Manifest.csv</t>
+          <t>NA73511_Evidence_Manifest.csv</t>
         </is>
       </c>
     </row>
@@ -1592,18 +1588,22 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>73212</t>
+          <t>73511</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Sight/obtain: Contracts: LCC-09-2022, Aust Care SO, Play Force</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr"/>
+          <t>Sight/obtain: Warnholtz invoice 001</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>744.30</t>
+        </is>
+      </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>NA73212_Evidence_Manifest.csv</t>
+          <t>NA73511_Evidence_Manifest.csv</t>
         </is>
       </c>
     </row>
@@ -1620,14 +1620,10 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Sight/obtain: INV-9747</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>2445.45</t>
-        </is>
-      </c>
+          <t>Sight/obtain: PCard/reimbursement receipts (net population)</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr"/>
       <c r="E46" s="4" t="inlineStr">
         <is>
           <t>NA73511_Evidence_Manifest.csv</t>
@@ -1647,12 +1643,12 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Sight/obtain: Warnholtz invoice 001</t>
+          <t>Sight/obtain: Hoffmann 18-Oct-2025 receipt</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>744.30</t>
+          <t>4.18</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
@@ -1674,10 +1670,14 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Sight/obtain: PCard/reimbursement receipts (net population)</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr"/>
+          <t>Sight/obtain: Finance FBT 50/50 batches (GJ076295 GJ076539 AP003647 AP003682 AP003801)</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
           <t>NA73511_Evidence_Manifest.csv</t>
@@ -1692,22 +1692,22 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>73511</t>
+          <t>73512</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Sight/obtain: Hoffmann 18-Oct-2025 receipt</t>
+          <t>Sight/obtain: 12052026 Preussner receipt</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>4.18</t>
+          <t>27.79</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>NA73511_Evidence_Manifest.csv</t>
+          <t>NA73512_Evidence_Manifest.csv</t>
         </is>
       </c>
     </row>
@@ -1719,22 +1719,22 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>73511</t>
+          <t>73512</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Sight/obtain: Finance FBT 50/50 batches (GJ076295 GJ076539 AP003647 AP003682 AP003801)</t>
+          <t>Sight/obtain: Quote 5468 vendor invoice</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1656.50</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>NA73511_Evidence_Manifest.csv</t>
+          <t>NA73512_Evidence_Manifest.csv</t>
         </is>
       </c>
     </row>
@@ -1751,14 +1751,10 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Sight/obtain: 12052026 Preussner receipt</t>
-        </is>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>27.79</t>
-        </is>
-      </c>
+          <t>Sight/obtain: Salisnew direct claims x6</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr"/>
       <c r="E51" s="4" t="inlineStr">
         <is>
           <t>NA73512_Evidence_Manifest.csv</t>
@@ -1778,14 +1774,10 @@
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Sight/obtain: Quote 5468 vendor invoice</t>
-        </is>
-      </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>1656.50</t>
-        </is>
-      </c>
+          <t>Sight/obtain: micro-line population refs 1179861-1211218</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr"/>
       <c r="E52" s="4" t="inlineStr">
         <is>
           <t>NA73512_Evidence_Manifest.csv</t>
@@ -1800,18 +1792,18 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>73512</t>
+          <t>73544</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Sight/obtain: Salisnew direct claims x6</t>
+          <t>Sight/obtain: OIR TE004236 source receipt</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr"/>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>NA73512_Evidence_Manifest.csv</t>
+          <t>NA73544_Evidence_Manifest.csv</t>
         </is>
       </c>
     </row>
@@ -1823,66 +1815,20 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>73512</t>
+          <t>73544</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Sight/obtain: micro-line population refs 1179861-1211218</t>
-        </is>
-      </c>
-      <c r="D54" s="4" t="inlineStr"/>
+          <t>Sight/obtain: Healthy Land &amp; Water tax invoice (BAL)</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>1767.00</t>
+        </is>
+      </c>
       <c r="E54" s="4" t="inlineStr">
-        <is>
-          <t>NA73512_Evidence_Manifest.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="7" t="inlineStr">
-        <is>
-          <t>EVIDENCE</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="inlineStr">
-        <is>
-          <t>73544</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>Sight/obtain: OIR TE004236 source receipt</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="inlineStr"/>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>NA73544_Evidence_Manifest.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="7" t="inlineStr">
-        <is>
-          <t>EVIDENCE</t>
-        </is>
-      </c>
-      <c r="B56" s="4" t="inlineStr">
-        <is>
-          <t>73544</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>Sight/obtain: Healthy Land &amp; Water tax invoice (BAL)</t>
-        </is>
-      </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>1767.00</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
         <is>
           <t>NA73544_Evidence_Manifest.csv</t>
         </is>

</xml_diff>